<commit_message>
Add VCI FVTPL/AFS composition data (4y + 8q + Q1/2026) and re-run analysis
Collected VCI's proprietary-trading asset composition from BCTC notes
(combined note "4. Các khoản đầu tư tài chính"), reconciled exactly
against source totals for every period. Re-ran the securities pipeline
so the FVTPL revenue driver now uses the real composition (CAPM-consistent)
instead of the assumed 35/30/35 mix. Also gitignore BCTC_PDF/ (raw source
PDFs, too large for git).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Bao cao/VCI/VCI_Model_2026-07-11.xlsx
+++ b/Bao cao/VCI/VCI_Model_2026-07-11.xlsx
@@ -25,6 +25,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_PE_PB_History" sheetId="16" state="visible" r:id="rId16"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_Segment_Quarterly" sheetId="17" state="visible" r:id="rId17"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_Peer_Benchmark" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16_FVTPL_Composition" sheetId="19" state="visible" r:id="rId19"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -172,7 +173,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -244,6 +245,9 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -11478,7 +11482,7 @@
         </is>
       </c>
       <c r="B26" s="8" t="n">
-        <v>0.0103</v>
+        <v>0.0104</v>
       </c>
       <c r="C26" s="7" t="n"/>
     </row>
@@ -11608,19 +11612,19 @@
         </is>
       </c>
       <c r="B4" s="13" t="n">
-        <v>-73.90000000000001</v>
+        <v>-139.4</v>
       </c>
       <c r="C4" s="13" t="n">
-        <v>-36.9</v>
+        <v>-69.7</v>
       </c>
       <c r="D4" s="13" t="n">
         <v>0</v>
       </c>
       <c r="E4" s="13" t="n">
-        <v>36.9</v>
+        <v>69.7</v>
       </c>
       <c r="F4" s="13" t="n">
-        <v>73.90000000000001</v>
+        <v>139.4</v>
       </c>
     </row>
     <row r="5">
@@ -11630,19 +11634,19 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>-0.042</v>
+        <v>-0.079</v>
       </c>
       <c r="C5" s="5" t="n">
-        <v>-0.021</v>
+        <v>-0.039</v>
       </c>
       <c r="D5" s="5" t="n">
         <v>0</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>0.021</v>
+        <v>0.039</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.042</v>
+        <v>0.079</v>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
@@ -12980,7 +12984,7 @@
       </c>
       <c r="B2" s="49" t="inlineStr">
         <is>
-          <t>Công ty Cổ phần Chứng khoán Vietcap vận hành mô hình 5 mảng: Môi giới, Cho vay Margin, Tự doanh (FVTPL), IB+Lưu ký, Quản lý quỹ. Mảng đóng góp lớn nhất hiện tại: Cho vay Margin (42.8% DT).</t>
+          <t>Công ty Cổ phần Chứng khoán Vietcap vận hành mô hình 5 mảng: Môi giới, Cho vay Margin, Tự doanh (FVTPL), IB+Lưu ký, Quản lý quỹ. Mảng đóng góp lớn nhất hiện tại: Cho vay Margin (42.5% DT).</t>
         </is>
       </c>
       <c r="C2" s="7" t="inlineStr">
@@ -13014,7 +13018,7 @@
       </c>
       <c r="B4" s="49" t="inlineStr">
         <is>
-          <t>Upside +25.7% so với giá hiện tại theo mô hình P/B (60%) + P/E (40%).</t>
+          <t>Upside +25.8% so với giá hiện tại theo mô hình P/B (60%) + P/E (40%).</t>
         </is>
       </c>
       <c r="C4" s="7" t="inlineStr">
@@ -13134,13 +13138,13 @@
         <v>4980.201525108</v>
       </c>
       <c r="G2" s="23" t="n">
-        <v>3633.4</v>
+        <v>3662.2</v>
       </c>
       <c r="H2" s="23" t="n">
-        <v>3175.8</v>
+        <v>3217.8</v>
       </c>
       <c r="I2" s="23" t="n">
-        <v>3404.8</v>
+        <v>3449.7</v>
       </c>
     </row>
     <row r="3">
@@ -13165,13 +13169,13 @@
         <v>1341.954507258</v>
       </c>
       <c r="G3" s="23" t="n">
-        <v>1457.6</v>
+        <v>1466.5</v>
       </c>
       <c r="H3" s="23" t="n">
-        <v>1301.6</v>
+        <v>1318.8</v>
       </c>
       <c r="I3" s="23" t="n">
-        <v>1395.5</v>
+        <v>1413.9</v>
       </c>
     </row>
     <row r="4">
@@ -13196,13 +13200,13 @@
         <v>1165</v>
       </c>
       <c r="G4" s="23" t="n">
-        <v>1265</v>
+        <v>1273</v>
       </c>
       <c r="H4" s="23" t="n">
-        <v>1130</v>
+        <v>1145</v>
       </c>
       <c r="I4" s="23" t="n">
-        <v>1211</v>
+        <v>1227</v>
       </c>
     </row>
     <row r="5">
@@ -13227,13 +13231,13 @@
         <v>15630</v>
       </c>
       <c r="G5" s="23" t="n">
-        <v>16642</v>
+        <v>16649</v>
       </c>
       <c r="H5" s="23" t="n">
-        <v>17546</v>
+        <v>17564</v>
       </c>
       <c r="I5" s="23" t="n">
-        <v>18515</v>
+        <v>18546</v>
       </c>
     </row>
     <row r="6">
@@ -13258,13 +13262,13 @@
         <v>18009.896539949</v>
       </c>
       <c r="G6" s="23" t="n">
-        <v>19175.976539949</v>
+        <v>19183.096539949</v>
       </c>
       <c r="H6" s="23" t="n">
-        <v>20217.256539949</v>
+        <v>20238.136539949</v>
       </c>
       <c r="I6" s="23" t="n">
-        <v>21333.656539949</v>
+        <v>21369.256539949</v>
       </c>
     </row>
     <row r="7">
@@ -13289,13 +13293,13 @@
         <v>7.45</v>
       </c>
       <c r="G7" s="53" t="n">
-        <v>7.6</v>
+        <v>7.64</v>
       </c>
       <c r="H7" s="53" t="n">
-        <v>6.44</v>
+        <v>6.52</v>
       </c>
       <c r="I7" s="53" t="n">
-        <v>6.54</v>
+        <v>6.62</v>
       </c>
     </row>
     <row r="8">
@@ -13320,13 +13324,13 @@
         <v>20.99</v>
       </c>
       <c r="G8" s="34" t="n">
-        <v>19.33</v>
+        <v>19.21</v>
       </c>
       <c r="H8" s="34" t="n">
-        <v>21.64</v>
+        <v>21.35</v>
       </c>
       <c r="I8" s="34" t="n">
-        <v>20.19</v>
+        <v>19.93</v>
       </c>
     </row>
     <row r="9">
@@ -15570,6 +15574,876 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L34"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="3" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="13" customWidth="1" min="14" max="14"/>
+    <col width="13" customWidth="1" min="15" max="15"/>
+    <col width="13" customWidth="1" min="16" max="16"/>
+    <col width="13" customWidth="1" min="17" max="17"/>
+    <col width="13" customWidth="1" min="18" max="18"/>
+    <col width="13" customWidth="1" min="19" max="19"/>
+    <col width="13" customWidth="1" min="20" max="20"/>
+    <col width="13" customWidth="1" min="21" max="21"/>
+    <col width="13" customWidth="1" min="22" max="22"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>CƠ CẤU &amp; HIỆU QUẢ DANH MỤC TỰ DOANH FVTPL/AFS — VCI</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Nguồn: thuyết minh BCTC hợp nhất (mục 'Tài sản tài chính ghi nhận thông qua lãi/lỗ FVTPL' / 'sẵn sàng để bán AFS'), trích trực tiếp — KHÔNG ước tính. Đơn vị: tỷ VND.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>1. CƠ CẤU DANH MỤC THEO NHÓM TÀI SẢN (Giá trị hợp lý, tỷ VND)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Nhóm tài sản</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>2022(N)</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>2023(N)</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>2024Q1</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>2024Q2</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>2024Q3</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>2024Q4</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>2025Q1</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>2025Q2</t>
+        </is>
+      </c>
+      <c r="J5" s="4" t="inlineStr">
+        <is>
+          <t>2025Q3</t>
+        </is>
+      </c>
+      <c r="K5" s="4" t="inlineStr">
+        <is>
+          <t>2025Q4</t>
+        </is>
+      </c>
+      <c r="L5" s="4" t="inlineStr">
+        <is>
+          <t>2026Q1</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="14" t="inlineStr">
+        <is>
+          <t>Cổ phiếu niêm yết/UPCoM</t>
+        </is>
+      </c>
+      <c r="B6" s="57" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="C6" s="57" t="n">
+        <v>122.1</v>
+      </c>
+      <c r="D6" s="57" t="n">
+        <v>412.6</v>
+      </c>
+      <c r="E6" s="57" t="n">
+        <v>753.8</v>
+      </c>
+      <c r="F6" s="57" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="G6" s="57" t="n">
+        <v>197.3</v>
+      </c>
+      <c r="H6" s="57" t="n">
+        <v>823.8</v>
+      </c>
+      <c r="I6" s="57" t="n">
+        <v>32.2</v>
+      </c>
+      <c r="J6" s="57" t="n">
+        <v>156.4</v>
+      </c>
+      <c r="K6" s="57" t="n">
+        <v>45</v>
+      </c>
+      <c r="L6" s="57" t="n">
+        <v>549.2</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="14" t="inlineStr">
+        <is>
+          <t>Cổ phiếu chưa niêm yết</t>
+        </is>
+      </c>
+      <c r="B7" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" s="57" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>Trái phiếu</t>
+        </is>
+      </c>
+      <c r="B8" s="57" t="n">
+        <v>598.6</v>
+      </c>
+      <c r="C8" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="57" t="n">
+        <v>40.6</v>
+      </c>
+      <c r="F8" s="57" t="n">
+        <v>452.5</v>
+      </c>
+      <c r="G8" s="57" t="n">
+        <v>628.6</v>
+      </c>
+      <c r="H8" s="57" t="n">
+        <v>271.9</v>
+      </c>
+      <c r="I8" s="57" t="n">
+        <v>713.5</v>
+      </c>
+      <c r="J8" s="57" t="n">
+        <v>443</v>
+      </c>
+      <c r="K8" s="57" t="n">
+        <v>2135.2</v>
+      </c>
+      <c r="L8" s="57" t="n">
+        <v>1316.9</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>Chứng chỉ quỹ (ETF+Quỹ mở)</t>
+        </is>
+      </c>
+      <c r="B9" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="57" t="n">
+        <v>213</v>
+      </c>
+      <c r="F9" s="57" t="n">
+        <v>21.6</v>
+      </c>
+      <c r="G9" s="57" t="n">
+        <v>20.4</v>
+      </c>
+      <c r="H9" s="57" t="n">
+        <v>99.59999999999999</v>
+      </c>
+      <c r="I9" s="57" t="n">
+        <v>31.4</v>
+      </c>
+      <c r="J9" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" s="57" t="n">
+        <v>57.7</v>
+      </c>
+      <c r="L9" s="57" t="n">
+        <v>173.2</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>Chứng chỉ tiền gửi</t>
+        </is>
+      </c>
+      <c r="B10" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="57" t="n">
+        <v>357</v>
+      </c>
+      <c r="E10" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" s="57" t="n">
+        <v>511.9</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>Tổng cộng</t>
+        </is>
+      </c>
+      <c r="B11" s="30">
+        <f>SUM(B6:B10)</f>
+        <v/>
+      </c>
+      <c r="C11" s="30">
+        <f>SUM(C6:C10)</f>
+        <v/>
+      </c>
+      <c r="D11" s="30">
+        <f>SUM(D6:D10)</f>
+        <v/>
+      </c>
+      <c r="E11" s="30">
+        <f>SUM(E6:E10)</f>
+        <v/>
+      </c>
+      <c r="F11" s="30">
+        <f>SUM(F6:F10)</f>
+        <v/>
+      </c>
+      <c r="G11" s="30">
+        <f>SUM(G6:G10)</f>
+        <v/>
+      </c>
+      <c r="H11" s="30">
+        <f>SUM(H6:H10)</f>
+        <v/>
+      </c>
+      <c r="I11" s="30">
+        <f>SUM(I6:I10)</f>
+        <v/>
+      </c>
+      <c r="J11" s="30">
+        <f>SUM(J6:J10)</f>
+        <v/>
+      </c>
+      <c r="K11" s="30">
+        <f>SUM(K6:K10)</f>
+        <v/>
+      </c>
+      <c r="L11" s="30">
+        <f>SUM(L6:L10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>2. LÃI/LỖ ĐÁNH GIÁ LẠI THEO NHÓM TÀI SẢN (tỷ VND, tại thời điểm báo cáo so với giá gốc)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Nhóm tài sản</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>2022(N)</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>2023(N)</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>2024Q1</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>2024Q2</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>2024Q3</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>2024Q4</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>2025Q1</t>
+        </is>
+      </c>
+      <c r="I15" s="4" t="inlineStr">
+        <is>
+          <t>2025Q2</t>
+        </is>
+      </c>
+      <c r="J15" s="4" t="inlineStr">
+        <is>
+          <t>2025Q3</t>
+        </is>
+      </c>
+      <c r="K15" s="4" t="inlineStr">
+        <is>
+          <t>2025Q4</t>
+        </is>
+      </c>
+      <c r="L15" s="4" t="inlineStr">
+        <is>
+          <t>2026Q1</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="14" t="inlineStr">
+        <is>
+          <t>Cổ phiếu niêm yết/UPCoM (ròng)</t>
+        </is>
+      </c>
+      <c r="B16" s="57" t="n">
+        <v>-1.6</v>
+      </c>
+      <c r="C16" s="57" t="n">
+        <v>-2.9</v>
+      </c>
+      <c r="D16" s="57" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="E16" s="57" t="n">
+        <v>-9</v>
+      </c>
+      <c r="F16" s="57" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G16" s="57" t="n">
+        <v>-3.9</v>
+      </c>
+      <c r="H16" s="57" t="n"/>
+      <c r="I16" s="57" t="n">
+        <v>-0.8</v>
+      </c>
+      <c r="J16" s="57" t="n">
+        <v>-4.2</v>
+      </c>
+      <c r="K16" s="57" t="n">
+        <v>-0.4</v>
+      </c>
+      <c r="L16" s="57" t="n">
+        <v>9.5</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="14" t="inlineStr">
+        <is>
+          <t>Cổ phiếu chưa niêm yết (ròng)</t>
+        </is>
+      </c>
+      <c r="B17" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" s="57" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="14" t="inlineStr">
+        <is>
+          <t>Trái phiếu (ròng)</t>
+        </is>
+      </c>
+      <c r="B18" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" s="57" t="n"/>
+      <c r="I18" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="J18" s="57" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="K18" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="L18" s="57" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="14" t="inlineStr">
+        <is>
+          <t>Chứng chỉ quỹ (ETF+Quỹ mở) (ròng)</t>
+        </is>
+      </c>
+      <c r="B19" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" s="57" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F19" s="57" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="G19" s="57" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="H19" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" s="57" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="J19" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="K19" s="57" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="L19" s="57" t="n">
+        <v>1.9</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="14" t="inlineStr">
+        <is>
+          <t>Chứng chỉ tiền gửi (ròng)</t>
+        </is>
+      </c>
+      <c r="B20" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="D20" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="I20" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="J20" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="K20" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="L20" s="57" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="inlineStr">
+        <is>
+          <t>3. DANH MỤC CỔ PHIẾU NIÊM YẾT CỤ THỂ ĐANG NẮM GIỮ (Giá trị hợp lý, tỷ VND)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Mã CP</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>2022(N)</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>2023(N)</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>2024(N)</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>2024Q2</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>2025(N)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="14" t="inlineStr">
+        <is>
+          <t>IDP</t>
+        </is>
+      </c>
+      <c r="B25" s="57" t="n">
+        <v>1617.9</v>
+      </c>
+      <c r="C25" s="57" t="n">
+        <v>2166.2</v>
+      </c>
+      <c r="D25" s="57" t="n">
+        <v>2117.6</v>
+      </c>
+      <c r="E25" s="57" t="n">
+        <v>2201.6</v>
+      </c>
+      <c r="F25" s="57" t="n">
+        <v>1945.2</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="14" t="inlineStr">
+        <is>
+          <t>KDH</t>
+        </is>
+      </c>
+      <c r="B26" s="57" t="n">
+        <v>357</v>
+      </c>
+      <c r="C26" s="57" t="n">
+        <v>1019</v>
+      </c>
+      <c r="D26" s="57" t="n">
+        <v>1183.8</v>
+      </c>
+      <c r="E26" s="57" t="n">
+        <v>1016.7</v>
+      </c>
+      <c r="F26" s="57" t="n">
+        <v>1065.2</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="14" t="inlineStr">
+        <is>
+          <t>MBB</t>
+        </is>
+      </c>
+      <c r="B27" s="57" t="n">
+        <v>176.1</v>
+      </c>
+      <c r="C27" s="57" t="n">
+        <v>246.6</v>
+      </c>
+      <c r="D27" s="57" t="n">
+        <v>12.3</v>
+      </c>
+      <c r="E27" s="57" t="n">
+        <v>222.6</v>
+      </c>
+      <c r="F27" s="57" t="n">
+        <v>450.9</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="14" t="inlineStr">
+        <is>
+          <t>MSN</t>
+        </is>
+      </c>
+      <c r="B28" s="57" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="C28" s="57" t="n">
+        <v>236.3</v>
+      </c>
+      <c r="D28" s="57" t="n"/>
+      <c r="E28" s="57" t="n">
+        <v>78</v>
+      </c>
+      <c r="F28" s="57" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="14" t="inlineStr">
+        <is>
+          <t>PNJ</t>
+        </is>
+      </c>
+      <c r="B29" s="57" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="C29" s="57" t="n">
+        <v>234.1</v>
+      </c>
+      <c r="D29" s="57" t="n"/>
+      <c r="E29" s="57" t="n">
+        <v>84.3</v>
+      </c>
+      <c r="F29" s="57" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="14" t="inlineStr">
+        <is>
+          <t>FPT</t>
+        </is>
+      </c>
+      <c r="B30" s="57" t="n"/>
+      <c r="C30" s="57" t="n">
+        <v>174.6</v>
+      </c>
+      <c r="D30" s="57" t="n">
+        <v>695.4</v>
+      </c>
+      <c r="E30" s="57" t="n">
+        <v>548.7</v>
+      </c>
+      <c r="F30" s="57" t="n">
+        <v>588.3</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="14" t="inlineStr">
+        <is>
+          <t>STB</t>
+        </is>
+      </c>
+      <c r="B31" s="57" t="n"/>
+      <c r="C31" s="57" t="n">
+        <v>109.2</v>
+      </c>
+      <c r="D31" s="57" t="n"/>
+      <c r="E31" s="57" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F31" s="57" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="14" t="inlineStr">
+        <is>
+          <t>MCH</t>
+        </is>
+      </c>
+      <c r="B32" s="57" t="n"/>
+      <c r="C32" s="57" t="n"/>
+      <c r="D32" s="57" t="n">
+        <v>569.7</v>
+      </c>
+      <c r="E32" s="57" t="n"/>
+      <c r="F32" s="57" t="n">
+        <v>2529.7</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="14" t="inlineStr">
+        <is>
+          <t>TDM</t>
+        </is>
+      </c>
+      <c r="B33" s="57" t="n"/>
+      <c r="C33" s="57" t="n"/>
+      <c r="D33" s="57" t="n">
+        <v>772.4</v>
+      </c>
+      <c r="E33" s="57" t="n">
+        <v>760</v>
+      </c>
+      <c r="F33" s="57" t="n">
+        <v>884.1</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="14" t="inlineStr">
+        <is>
+          <t>Khac</t>
+        </is>
+      </c>
+      <c r="B34" s="57" t="n">
+        <v>681.8</v>
+      </c>
+      <c r="C34" s="57" t="n">
+        <v>1556.6</v>
+      </c>
+      <c r="D34" s="57" t="n">
+        <v>1668.1</v>
+      </c>
+      <c r="E34" s="57" t="n">
+        <v>2060.4</v>
+      </c>
+      <c r="F34" s="57" t="n">
+        <v>2959.7</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -15619,7 +16493,7 @@
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>Fallback (manual)</t>
+          <t>Cache lần chạy trước (2026-07-11 19:01)</t>
         </is>
       </c>
     </row>
@@ -15758,7 +16632,7 @@
         </is>
       </c>
       <c r="C10" s="13" t="n">
-        <v>32119</v>
+        <v>32133</v>
       </c>
     </row>
     <row r="11">
@@ -15768,7 +16642,7 @@
         </is>
       </c>
       <c r="C11" s="13" t="n">
-        <v>18229</v>
+        <v>18344</v>
       </c>
     </row>
     <row r="12">
@@ -15801,7 +16675,7 @@
         </is>
       </c>
       <c r="C15" s="16" t="n">
-        <v>30730</v>
+        <v>30754</v>
       </c>
     </row>
     <row r="16">
@@ -15811,7 +16685,7 @@
         </is>
       </c>
       <c r="C16" s="5" t="n">
-        <v>0.257</v>
+        <v>0.258</v>
       </c>
     </row>
     <row r="17">
@@ -16279,17 +17153,17 @@
       <c r="E19" s="8" t="n"/>
       <c r="F19" s="8" t="n"/>
       <c r="G19" s="21" t="n">
-        <v>0.5</v>
+        <v>0.2007</v>
       </c>
       <c r="H19" s="21" t="n">
-        <v>0.5</v>
+        <v>0.2007</v>
       </c>
       <c r="I19" s="21" t="n">
-        <v>0.5</v>
+        <v>0.2007</v>
       </c>
       <c r="J19" s="20" t="inlineStr">
         <is>
-          <t>⚠ GIẢ ĐỊNH THỦ CÔNG — chưa có data/fvtpl_holdings/VCI.json (thuyết minh cơ cấu danh mục FVTPL chi tiết theo loại tài sản), nên dùng bảng giả định chung theo ticker/ngành. Mặc định chỉ mang tính khởi điểm — BẮT BUỘC điều chỉnh theo thuyết minh BCTC thực tế nếu có. Đối chiếu với dòng 'Hiệu suất Tự doanh THỰC TẾ lịch sử' bên dưới để hiệu chỉnh.</t>
+          <t>✓ CƠ CẤU THẬT — trích trực tiếp từ thuyết minh BCTC (data/fvtpl_holdings/VCI.json, kỳ gần nhất, xem sheet 16_FVTPL_Composition) — KHÔNG phải giả định. Cập nhật lại khi có kỳ báo cáo mới hơn (chạy lại quy trình thu thập dữ liệu FVTPL).</t>
         </is>
       </c>
     </row>
@@ -16305,17 +17179,17 @@
       <c r="E20" s="8" t="n"/>
       <c r="F20" s="8" t="n"/>
       <c r="G20" s="21" t="n">
-        <v>0.35</v>
+        <v>0.5162</v>
       </c>
       <c r="H20" s="21" t="n">
-        <v>0.35</v>
+        <v>0.5162</v>
       </c>
       <c r="I20" s="21" t="n">
-        <v>0.35</v>
+        <v>0.5162</v>
       </c>
       <c r="J20" s="20" t="inlineStr">
         <is>
-          <t>⚠ GIẢ ĐỊNH THỦ CÔNG — chưa có data/fvtpl_holdings/VCI.json (thuyết minh cơ cấu danh mục FVTPL chi tiết theo loại tài sản), nên dùng bảng giả định chung theo ticker/ngành. Mặc định chỉ mang tính khởi điểm — BẮT BUỘC điều chỉnh theo thuyết minh BCTC thực tế nếu có. Đối chiếu với dòng 'Hiệu suất Tự doanh THỰC TẾ lịch sử' bên dưới để hiệu chỉnh.</t>
+          <t>✓ CƠ CẤU THẬT — trích trực tiếp từ thuyết minh BCTC (data/fvtpl_holdings/VCI.json, kỳ gần nhất, xem sheet 16_FVTPL_Composition) — KHÔNG phải giả định. Cập nhật lại khi có kỳ báo cáo mới hơn (chạy lại quy trình thu thập dữ liệu FVTPL).</t>
         </is>
       </c>
     </row>
@@ -16331,17 +17205,17 @@
       <c r="E21" s="8" t="n"/>
       <c r="F21" s="8" t="n"/>
       <c r="G21" s="21" t="n">
-        <v>0.15</v>
+        <v>0.2832</v>
       </c>
       <c r="H21" s="21" t="n">
-        <v>0.15</v>
+        <v>0.2832</v>
       </c>
       <c r="I21" s="21" t="n">
-        <v>0.15</v>
+        <v>0.2832</v>
       </c>
       <c r="J21" s="20" t="inlineStr">
         <is>
-          <t>⚠ GIẢ ĐỊNH THỦ CÔNG — chưa có data/fvtpl_holdings/VCI.json (thuyết minh cơ cấu danh mục FVTPL chi tiết theo loại tài sản), nên dùng bảng giả định chung theo ticker/ngành. Mặc định chỉ mang tính khởi điểm — BẮT BUỘC điều chỉnh theo thuyết minh BCTC thực tế nếu có. Đối chiếu với dòng 'Hiệu suất Tự doanh THỰC TẾ lịch sử' bên dưới để hiệu chỉnh.</t>
+          <t>✓ CƠ CẤU THẬT — trích trực tiếp từ thuyết minh BCTC (data/fvtpl_holdings/VCI.json, kỳ gần nhất, xem sheet 16_FVTPL_Composition) — KHÔNG phải giả định. Cập nhật lại khi có kỳ báo cáo mới hơn (chạy lại quy trình thu thập dữ liệu FVTPL).</t>
         </is>
       </c>
     </row>
@@ -16400,7 +17274,7 @@
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
         <is>
-          <t>R_VNI — Biến động kỳ vọng VN-Index (%/năm)</t>
+          <t>R_VNI — Lợi suất kỳ vọng CP+Chứng chỉ quỹ (%/năm)</t>
         </is>
       </c>
       <c r="B24" s="8" t="n"/>
@@ -16409,17 +17283,17 @@
       <c r="E24" s="8" t="n"/>
       <c r="F24" s="8" t="n"/>
       <c r="G24" s="21" t="n">
-        <v>0.1</v>
+        <v>0.1437</v>
       </c>
       <c r="H24" s="21" t="n">
-        <v>0.1</v>
+        <v>0.1437</v>
       </c>
       <c r="I24" s="21" t="n">
-        <v>0.1</v>
+        <v>0.1437</v>
       </c>
       <c r="J24" s="20" t="inlineStr">
         <is>
-          <t>⚠ KHÔNG kiểm chứng được — kỳ vọng lợi suất tương lai mang tính chủ quan, không có "đúng/sai". Đối chiếu với COE (sheet 00_COE) hoặc quan điểm thị trường riêng khi điều chỉnh</t>
+          <t>✓ NHẤT QUÁN CAPM — dùng ĐÚNG COE (sheet 00_COE = Rf+β×ERP+α của chính ticker này) làm lợi suất kỳ vọng phần rủi ro cổ phiếu, thay vì con số 10% chủ quan trước đây — cùng suất chiết khấu với mô hình định giá.</t>
         </is>
       </c>
     </row>
@@ -18536,13 +19410,13 @@
         <v>16064.5</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>22431.9</v>
+        <v>22424.7</v>
       </c>
       <c r="H7" s="13" t="n">
-        <v>25550.6</v>
+        <v>25529.7</v>
       </c>
       <c r="I7" s="13" t="n">
-        <v>28049.2</v>
+        <v>28013.6</v>
       </c>
     </row>
     <row r="8">
@@ -18637,13 +19511,13 @@
         <v>18009.9</v>
       </c>
       <c r="G10" s="30" t="n">
-        <v>19176</v>
+        <v>19183.1</v>
       </c>
       <c r="H10" s="30" t="n">
-        <v>20217.3</v>
+        <v>20238.1</v>
       </c>
       <c r="I10" s="30" t="n">
-        <v>21333.7</v>
+        <v>21369.3</v>
       </c>
     </row>
     <row r="12">

</xml_diff>